<commit_message>
bugfix: empty choices in spreadsheets was not being detected.
If a spreadsheet has a missing activity / field  for land or water choices then it was supposed to trigger an error. Current logic was reassigning the activity from the row above in the spreadsheet if the activity was missing. Moved initialization of kids names and activities within the loop to reset name and activities back to empty strings after processing each row.

Updated several excel test files that all contained a single missing value for an activity to stop tests failing.

Changed new-excel-format.xlsx --> success-117-kids.xlsx to follow convention of file naming for test files.
</commit_message>
<xml_diff>
--- a/e2e/fixtures/new-format/error-147-kids.xlsx
+++ b/e2e/fixtures/new-format/error-147-kids.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darren/Projects/NY-Sheriff-Summer-Camp-Scheduler/e2e/fixtures/new-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB1652C-A4C1-6E4C-87C7-E38BA7A5CEE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C69B8B1-1DAB-9B4C-8C5B-A03C3C4B33B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="44800" windowHeight="25200" firstSheet="1" activeTab="1" xr2:uid="{B75E9CFD-F73C-4E0E-B330-6F712BC21BE5}"/>
   </bookViews>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6522" uniqueCount="1354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6523" uniqueCount="1354">
   <si>
     <t>Otsego</t>
   </si>
@@ -10250,7 +10250,9 @@
       <c r="AT28" s="26" t="s">
         <v>257</v>
       </c>
-      <c r="AU28" s="26"/>
+      <c r="AU28" s="26" t="s">
+        <v>148</v>
+      </c>
       <c r="AV28" s="26" t="s">
         <v>149</v>
       </c>

</xml_diff>

<commit_message>
chore: fix tests to match update excel data.
</commit_message>
<xml_diff>
--- a/e2e/fixtures/new-format/error-147-kids.xlsx
+++ b/e2e/fixtures/new-format/error-147-kids.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darren/Projects/NY-Sheriff-Summer-Camp-Scheduler/e2e/fixtures/new-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A18F3714-7227-FB4D-B2F9-927952155E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F474CB47-F46E-7B47-89BC-34AE52311666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="44800" windowHeight="25200" firstSheet="1" activeTab="1" xr2:uid="{B75E9CFD-F73C-4E0E-B330-6F712BC21BE5}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2433" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2433" uniqueCount="415">
   <si>
     <t>Otsego</t>
   </si>
@@ -1286,6 +1286,9 @@
   </si>
   <si>
     <t>Brave</t>
+  </si>
+  <si>
+    <t>Ted</t>
   </si>
 </sst>
 </file>
@@ -10370,7 +10373,7 @@
         <v>411</v>
       </c>
       <c r="F148" s="23" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G148" s="24" t="s">
         <v>145</v>

</xml_diff>